<commit_message>
feat(media): PNG-only photo uploads, checked before a bulk import
File pickers accept PNG only; the import reads the first bytes of each .png to catch renamed files, and the template and on-page guidance say PNG.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LEp9pf58S2q2682KyDvfPv
</commit_message>
<xml_diff>
--- a/public/templates/rogueon-products-template.xlsx
+++ b/public/templates/rogueon-products-template.xlsx
@@ -561,8 +561,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
-      <c r="K2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -592,10 +590,6 @@
       <c r="G3" t="n">
         <v>12</v>
       </c>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
-      <c r="J3" t="inlineStr"/>
-      <c r="K3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -625,10 +619,6 @@
       <c r="G4" t="n">
         <v>20</v>
       </c>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -672,8 +662,6 @@
           <t>yes</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr"/>
-      <c r="K5" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -710,9 +698,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -727,9 +713,7 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
@@ -786,9 +770,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
@@ -824,9 +806,7 @@
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" t="inlineStr"/>
-    </row>
+    <row r="20"/>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
@@ -844,21 +824,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t xml:space="preserve">  photos/Project Requiem Zipup/1.jpg, 2.jpg        (general photos)</t>
+          <t xml:space="preserve">  photos/Project Requiem Zipup/1.png, 2.png        (general photos)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t xml:space="preserve">  photos/Project Requiem Zipup/Grey/1.jpg, 2.jpg   (photos of the grey one)</t>
+          <t xml:space="preserve">  photos/Project Requiem Zipup/Grey/1.png, 2.png   (photos of the grey one)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t xml:space="preserve">  photos/Project Requiem Zipup/Black/1.jpg</t>
+          <t xml:space="preserve">  photos/Project Requiem Zipup/Black/1.png</t>
         </is>
       </c>
     </row>
@@ -872,13 +852,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Number the files in the order they should show. JPEG, PNG or WebP, up to 8 MB each, 20 per product.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr"/>
-    </row>
+          <t>Number the files in the order they should show. Photos must be PNG (JPEG and other formats are refused), up to 8 MB each, 20 per product.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>

</xml_diff>